<commit_message>
Confirm EXPRESS_MAXIMUM supplier name has no space after "PT."
User confirmed the correct value is "PT.EXPRESS MAXIMUM" (no space),
matching the newest sample's reference -- the two previously-verified
samples' reference cells that had "PT. EXPRESS MAXIMUM" (with a space)
were the actual inconsistency. Updated the hardcoded header value and
the registry display label to match, and corrected the supplier cell
in all three test_samples/EXPRESS_MAXIMUM reference copies so the
regression harness reflects the confirmed convention.

Re-verified with run_regression.py: all 3 EXPRESS_MAXIMUM samples and
the full 13-supplier suite still pass 100%.
</commit_message>
<xml_diff>
--- a/test_samples/EXPRESS_MAXIMUM/sample3_ref.xlsx
+++ b/test_samples/EXPRESS_MAXIMUM/sample3_ref.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PT. EXPRESS MAXIMUM</t>
+          <t>PT.EXPRESS MAXIMUM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">

</xml_diff>